<commit_message>
Primeiro commit - Comex Bot
</commit_message>
<xml_diff>
--- a/comex_resultado.xlsx
+++ b/comex_resultado.xlsx
@@ -498,7 +498,7 @@
         <v>424630</v>
       </c>
       <c r="H2" t="n">
-        <v>250000</v>
+        <v>10.8695652173913</v>
       </c>
       <c r="I2" t="n">
         <v>1698.52</v>
@@ -539,7 +539,7 @@
         <v>298396</v>
       </c>
       <c r="H3" t="n">
-        <v>192000</v>
+        <v>8.347826086956522</v>
       </c>
       <c r="I3" t="n">
         <v>1554.145833333333</v>
@@ -580,7 +580,7 @@
         <v>143138</v>
       </c>
       <c r="H4" t="n">
-        <v>96000</v>
+        <v>4.173913043478261</v>
       </c>
       <c r="I4" t="n">
         <v>1491.020833333333</v>
@@ -621,7 +621,7 @@
         <v>43246</v>
       </c>
       <c r="H5" t="n">
-        <v>24000</v>
+        <v>1.043478260869565</v>
       </c>
       <c r="I5" t="n">
         <v>1801.916666666667</v>
@@ -662,7 +662,7 @@
         <v>33329</v>
       </c>
       <c r="H6" t="n">
-        <v>20000</v>
+        <v>0.8695652173913043</v>
       </c>
       <c r="I6" t="n">
         <v>1666.45</v>

</xml_diff>

<commit_message>
Atualiza calculo de conteineres
</commit_message>
<xml_diff>
--- a/comex_resultado.xlsx
+++ b/comex_resultado.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,11 @@
           <t>US$/ton</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Contêiner</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -498,10 +503,13 @@
         <v>424630</v>
       </c>
       <c r="H2" t="n">
-        <v>10.8695652173913</v>
+        <v>250000</v>
       </c>
       <c r="I2" t="n">
         <v>1698.52</v>
+      </c>
+      <c r="J2" t="n">
+        <v>10.8695652173913</v>
       </c>
     </row>
     <row r="3">
@@ -539,10 +547,13 @@
         <v>298396</v>
       </c>
       <c r="H3" t="n">
-        <v>8.347826086956522</v>
+        <v>192000</v>
       </c>
       <c r="I3" t="n">
         <v>1554.145833333333</v>
+      </c>
+      <c r="J3" t="n">
+        <v>8.347826086956522</v>
       </c>
     </row>
     <row r="4">
@@ -580,10 +591,13 @@
         <v>143138</v>
       </c>
       <c r="H4" t="n">
-        <v>4.173913043478261</v>
+        <v>96000</v>
       </c>
       <c r="I4" t="n">
         <v>1491.020833333333</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4.173913043478261</v>
       </c>
     </row>
     <row r="5">
@@ -621,10 +635,13 @@
         <v>43246</v>
       </c>
       <c r="H5" t="n">
-        <v>1.043478260869565</v>
+        <v>24000</v>
       </c>
       <c r="I5" t="n">
         <v>1801.916666666667</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.043478260869565</v>
       </c>
     </row>
     <row r="6">
@@ -662,10 +679,13 @@
         <v>33329</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8695652173913043</v>
+        <v>20000</v>
       </c>
       <c r="I6" t="n">
         <v>1666.45</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.8695652173913043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>